<commit_message>
Update exported spreadsheet after issue flow changes
</commit_message>
<xml_diff>
--- a/var/exports/controle_saidas.xlsx
+++ b/var/exports/controle_saidas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1053,6 +1053,122 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-02-19 19:23</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>adfgadg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>012.001.004</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ABRAÇADEIRA NYLON BRANCA 40 CM</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-02-19 19:32</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>fewqfeq</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>fwqefweq</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>012.001.001</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ABRAÇADEIRA NYLON BRANCA 15 CM</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>23</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-02-19 19:35</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>vfevf</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>bdsbadb</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>012.001.004</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ABRAÇADEIRA NYLON BRANCA 40 CM</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>